<commit_message>
Fix the sesssion import sheet so that it is clear what the columns actually map to
</commit_message>
<xml_diff>
--- a/public/examples/session_import.xlsx
+++ b/public/examples/session_import.xlsx
@@ -8,7 +8,7 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId2"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t xml:space="preserve">Area</t>
   </si>
@@ -34,16 +34,13 @@
     <t xml:space="preserve">Format</t>
   </si>
   <si>
-    <t xml:space="preserve">GoH/Participant Dependent?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Signups?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Additional instructions for signups</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tags</t>
+    <t xml:space="preserve">GoH Notes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open for Interest</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Interest Instructions</t>
   </si>
   <si>
     <t xml:space="preserve">Notes</t>
@@ -79,6 +76,7 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -100,12 +98,14 @@
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="0"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="0"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -150,20 +150,24 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -179,70 +183,174 @@
 </styleSheet>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office">
+  <a:themeElements>
+    <a:clrScheme name="LibreOffice">
+      <a:dk1>
+        <a:srgbClr val="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:srgbClr val="ffffff"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="000000"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="ffffff"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="18a303"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="0369a3"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="a33e03"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8e03a3"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="c99c00"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="c9211e"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000ee"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="551a8b"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme>
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="29.26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="57.26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="29.26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="57.26"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="14.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+    <row r="1" customFormat="false" ht="14.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
+    </row>
+    <row r="2" customFormat="false" ht="25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="2" customFormat="false" ht="23.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="B2" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="C2" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="D2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="E2" s="4"/>
+      <c r="F2" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="G2" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="G2" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="I2" s="2"/>
+      <c r="H2" s="3"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="C2">
+  <conditionalFormatting sqref="E2 C2">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min" val="0"/>
@@ -253,18 +361,18 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2" type="list">
       <formula1>"Panel,Presentation,Demonstration,Workshop,Discussion,Interview,Dialogue,Meetup,Other (add to notes)"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="F2" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="F2" type="list">
       <formula1>"Yes,No"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.025" bottom="1.025" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="1" scale="100" firstPageNumber="1" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader>&amp;C&amp;A</oddHeader>
     <oddFooter>&amp;CPage &amp;P</oddFooter>

</xml_diff>